<commit_message>
Primeira versão do America Lanche
</commit_message>
<xml_diff>
--- a/static/cardapio.xlsx
+++ b/static/cardapio.xlsx
@@ -9,10 +9,11 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28770" windowHeight="11880"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28770" windowHeight="11880" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Cardapio" sheetId="1" r:id="rId1"/>
+    <sheet name="Adicionais" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="86">
   <si>
     <t>Pão, hambúrguer, presunto, queijo, bacon, calabresa, ovo frito, frango, coração, alface, tomate, milho, ervilha, batata palha</t>
   </si>
@@ -279,6 +280,9 @@
   </si>
   <si>
     <t>preco</t>
+  </si>
+  <si>
+    <t>adicionais</t>
   </si>
 </sst>
 </file>
@@ -410,7 +414,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -428,6 +432,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -745,32 +758,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="C1" s="14" t="s">
+      <c r="C1" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="17" t="s">
         <v>84</v>
       </c>
-      <c r="E1" s="14" t="s">
+      <c r="E1" s="17" t="s">
         <v>83</v>
       </c>
       <c r="F1" s="2"/>
     </row>
     <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B2" s="2"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
       <c r="F2" s="2"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B3" s="1"/>
-      <c r="C3" s="15"/>
-      <c r="D3" s="15"/>
-      <c r="E3" s="15"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
     </row>
     <row r="4" spans="1:6" ht="60" x14ac:dyDescent="0.25">
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="19" t="s">
         <v>18</v>
       </c>
       <c r="C4" s="5" t="s">
@@ -784,7 +797,7 @@
       </c>
     </row>
     <row r="5" spans="1:6" ht="45" x14ac:dyDescent="0.25">
-      <c r="B5" s="16"/>
+      <c r="B5" s="19"/>
       <c r="C5" s="5" t="s">
         <v>25</v>
       </c>
@@ -796,7 +809,7 @@
       </c>
     </row>
     <row r="6" spans="1:6" ht="45" x14ac:dyDescent="0.25">
-      <c r="B6" s="16"/>
+      <c r="B6" s="19"/>
       <c r="C6" s="5" t="s">
         <v>26</v>
       </c>
@@ -808,7 +821,7 @@
       </c>
     </row>
     <row r="7" spans="1:6" ht="45" x14ac:dyDescent="0.25">
-      <c r="B7" s="16"/>
+      <c r="B7" s="19"/>
       <c r="C7" s="5" t="s">
         <v>53</v>
       </c>
@@ -820,7 +833,7 @@
       </c>
     </row>
     <row r="8" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="B8" s="16"/>
+      <c r="B8" s="19"/>
       <c r="C8" s="5" t="s">
         <v>52</v>
       </c>
@@ -832,7 +845,7 @@
       </c>
     </row>
     <row r="9" spans="1:6" ht="45" x14ac:dyDescent="0.25">
-      <c r="B9" s="16"/>
+      <c r="B9" s="19"/>
       <c r="C9" s="5" t="s">
         <v>51</v>
       </c>
@@ -844,7 +857,7 @@
       </c>
     </row>
     <row r="10" spans="1:6" ht="45" x14ac:dyDescent="0.25">
-      <c r="B10" s="16"/>
+      <c r="B10" s="19"/>
       <c r="C10" s="5" t="s">
         <v>50</v>
       </c>
@@ -856,7 +869,7 @@
       </c>
     </row>
     <row r="11" spans="1:6" ht="45" x14ac:dyDescent="0.25">
-      <c r="B11" s="16"/>
+      <c r="B11" s="19"/>
       <c r="C11" s="5" t="s">
         <v>56</v>
       </c>
@@ -868,7 +881,7 @@
       </c>
     </row>
     <row r="12" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="B12" s="16"/>
+      <c r="B12" s="19"/>
       <c r="C12" s="5" t="s">
         <v>46</v>
       </c>
@@ -880,7 +893,7 @@
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B13" s="16"/>
+      <c r="B13" s="19"/>
       <c r="C13" s="5" t="s">
         <v>47</v>
       </c>
@@ -892,7 +905,7 @@
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B14" s="16"/>
+      <c r="B14" s="19"/>
       <c r="C14" s="5" t="s">
         <v>48</v>
       </c>
@@ -904,7 +917,7 @@
       </c>
     </row>
     <row r="15" spans="1:6" ht="45" x14ac:dyDescent="0.25">
-      <c r="B15" s="16"/>
+      <c r="B15" s="19"/>
       <c r="C15" s="5" t="s">
         <v>49</v>
       </c>
@@ -924,7 +937,7 @@
       <c r="F16" s="3"/>
     </row>
     <row r="17" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="B17" s="16" t="s">
+      <c r="B17" s="19" t="s">
         <v>19</v>
       </c>
       <c r="C17" s="5" t="s">
@@ -938,7 +951,7 @@
       </c>
     </row>
     <row r="18" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="B18" s="16"/>
+      <c r="B18" s="19"/>
       <c r="C18" s="5" t="s">
         <v>43</v>
       </c>
@@ -950,7 +963,7 @@
       </c>
     </row>
     <row r="19" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="B19" s="16"/>
+      <c r="B19" s="19"/>
       <c r="C19" s="5" t="s">
         <v>45</v>
       </c>
@@ -983,7 +996,7 @@
       <c r="E30" s="4"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B31" s="9" t="s">
+      <c r="B31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="C31" s="5" t="s">
@@ -995,7 +1008,7 @@
       <c r="E31" s="5"/>
     </row>
     <row r="32" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="B32" s="10"/>
+      <c r="B32" s="13"/>
       <c r="C32" s="5" t="s">
         <v>40</v>
       </c>
@@ -1005,7 +1018,7 @@
       <c r="E32" s="5"/>
     </row>
     <row r="33" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="B33" s="10"/>
+      <c r="B33" s="13"/>
       <c r="C33" s="5" t="s">
         <v>39</v>
       </c>
@@ -1015,7 +1028,7 @@
       <c r="E33" s="5"/>
     </row>
     <row r="34" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="B34" s="10"/>
+      <c r="B34" s="13"/>
       <c r="C34" s="5" t="s">
         <v>38</v>
       </c>
@@ -1025,7 +1038,7 @@
       <c r="E34" s="5"/>
     </row>
     <row r="35" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="B35" s="10"/>
+      <c r="B35" s="13"/>
       <c r="C35" s="5" t="s">
         <v>37</v>
       </c>
@@ -1035,7 +1048,7 @@
       <c r="E35" s="5"/>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B36" s="10"/>
+      <c r="B36" s="13"/>
       <c r="C36" s="5" t="s">
         <v>36</v>
       </c>
@@ -1045,7 +1058,7 @@
       <c r="E36" s="5"/>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B37" s="10"/>
+      <c r="B37" s="13"/>
       <c r="C37" s="5" t="s">
         <v>35</v>
       </c>
@@ -1056,7 +1069,7 @@
     </row>
     <row r="38" spans="1:6" ht="33.75" x14ac:dyDescent="0.5">
       <c r="A38" s="2"/>
-      <c r="B38" s="11"/>
+      <c r="B38" s="14"/>
       <c r="C38" s="5" t="s">
         <v>34</v>
       </c>
@@ -1067,7 +1080,7 @@
       <c r="F38" s="2"/>
     </row>
     <row r="39" spans="1:6" ht="75" x14ac:dyDescent="0.25">
-      <c r="B39" s="9" t="s">
+      <c r="B39" s="12" t="s">
         <v>22</v>
       </c>
       <c r="C39" s="5" t="s">
@@ -1081,7 +1094,7 @@
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B40" s="10"/>
+      <c r="B40" s="13"/>
       <c r="C40" s="5" t="s">
         <v>32</v>
       </c>
@@ -1093,7 +1106,7 @@
       </c>
     </row>
     <row r="41" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="11"/>
+      <c r="B41" s="14"/>
       <c r="C41" s="5" t="s">
         <v>31</v>
       </c>
@@ -1106,7 +1119,7 @@
     </row>
     <row r="42" spans="1:6" ht="33.75" x14ac:dyDescent="0.25">
       <c r="A42" s="4"/>
-      <c r="B42" s="9" t="s">
+      <c r="B42" s="12" t="s">
         <v>23</v>
       </c>
       <c r="C42" s="5" t="s">
@@ -1119,7 +1132,7 @@
       <c r="F42" s="4"/>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B43" s="10"/>
+      <c r="B43" s="13"/>
       <c r="C43" s="5" t="s">
         <v>58</v>
       </c>
@@ -1129,7 +1142,7 @@
       <c r="E43" s="5"/>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B44" s="10"/>
+      <c r="B44" s="13"/>
       <c r="C44" s="5" t="s">
         <v>59</v>
       </c>
@@ -1139,7 +1152,7 @@
       <c r="E44" s="5"/>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B45" s="10"/>
+      <c r="B45" s="13"/>
       <c r="C45" s="5" t="s">
         <v>60</v>
       </c>
@@ -1149,7 +1162,7 @@
       <c r="E45" s="5"/>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B46" s="10"/>
+      <c r="B46" s="13"/>
       <c r="C46" s="5" t="s">
         <v>61</v>
       </c>
@@ -1159,7 +1172,7 @@
       <c r="E46" s="5"/>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B47" s="10"/>
+      <c r="B47" s="13"/>
       <c r="C47" s="5" t="s">
         <v>62</v>
       </c>
@@ -1169,7 +1182,7 @@
       <c r="E47" s="5"/>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B48" s="10"/>
+      <c r="B48" s="13"/>
       <c r="C48" s="5" t="s">
         <v>63</v>
       </c>
@@ -1179,7 +1192,7 @@
       <c r="E48" s="5"/>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B49" s="10"/>
+      <c r="B49" s="13"/>
       <c r="C49" s="5" t="s">
         <v>64</v>
       </c>
@@ -1189,7 +1202,7 @@
       <c r="E49" s="5"/>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B50" s="10"/>
+      <c r="B50" s="13"/>
       <c r="C50" s="5" t="s">
         <v>30</v>
       </c>
@@ -1199,7 +1212,7 @@
       <c r="E50" s="5"/>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B51" s="10"/>
+      <c r="B51" s="13"/>
       <c r="C51" s="5" t="s">
         <v>65</v>
       </c>
@@ -1209,7 +1222,7 @@
       <c r="E51" s="5"/>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B52" s="10"/>
+      <c r="B52" s="13"/>
       <c r="C52" s="5" t="s">
         <v>66</v>
       </c>
@@ -1219,7 +1232,7 @@
       <c r="E52" s="5"/>
     </row>
     <row r="53" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="B53" s="11"/>
+      <c r="B53" s="14"/>
       <c r="C53" s="5" t="s">
         <v>29</v>
       </c>
@@ -1239,7 +1252,7 @@
       <c r="E56" s="4"/>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B57" s="9" t="s">
+      <c r="B57" s="12" t="s">
         <v>24</v>
       </c>
       <c r="C57" s="5" t="s">
@@ -1251,7 +1264,7 @@
       <c r="E57" s="5"/>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B58" s="10"/>
+      <c r="B58" s="13"/>
       <c r="C58" s="5" t="s">
         <v>27</v>
       </c>
@@ -1261,7 +1274,7 @@
       <c r="E58" s="5"/>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B59" s="10"/>
+      <c r="B59" s="13"/>
       <c r="C59" s="5" t="s">
         <v>67</v>
       </c>
@@ -1271,7 +1284,7 @@
       <c r="E59" s="5"/>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B60" s="10"/>
+      <c r="B60" s="13"/>
       <c r="C60" s="5" t="s">
         <v>68</v>
       </c>
@@ -1281,7 +1294,7 @@
       <c r="E60" s="5"/>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B61" s="10"/>
+      <c r="B61" s="13"/>
       <c r="C61" s="5" t="s">
         <v>69</v>
       </c>
@@ -1291,7 +1304,7 @@
       <c r="E61" s="5"/>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B62" s="10"/>
+      <c r="B62" s="13"/>
       <c r="C62" s="5" t="s">
         <v>70</v>
       </c>
@@ -1301,7 +1314,7 @@
       <c r="E62" s="5"/>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B63" s="10"/>
+      <c r="B63" s="13"/>
       <c r="C63" t="s">
         <v>72</v>
       </c>
@@ -1311,7 +1324,7 @@
       <c r="E63" s="5"/>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B64" s="11"/>
+      <c r="B64" s="14"/>
       <c r="C64" s="5" t="s">
         <v>71</v>
       </c>
@@ -1321,7 +1334,7 @@
       <c r="E64" s="5"/>
     </row>
     <row r="67" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B67" s="12" t="s">
+      <c r="B67" s="15" t="s">
         <v>20</v>
       </c>
       <c r="C67" s="6" t="s">
@@ -1333,7 +1346,7 @@
       <c r="E67" s="5"/>
     </row>
     <row r="68" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B68" s="13"/>
+      <c r="B68" s="16"/>
       <c r="C68" s="5" t="s">
         <v>74</v>
       </c>
@@ -1343,7 +1356,7 @@
       <c r="E68" s="5"/>
     </row>
     <row r="69" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B69" s="13"/>
+      <c r="B69" s="16"/>
       <c r="C69" s="5" t="s">
         <v>42</v>
       </c>
@@ -1353,7 +1366,7 @@
       <c r="E69" s="5"/>
     </row>
     <row r="70" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B70" s="13"/>
+      <c r="B70" s="16"/>
       <c r="C70" s="5" t="s">
         <v>76</v>
       </c>
@@ -1363,7 +1376,7 @@
       <c r="E70" s="5"/>
     </row>
     <row r="71" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B71" s="13"/>
+      <c r="B71" s="16"/>
       <c r="C71" s="5" t="s">
         <v>81</v>
       </c>
@@ -1373,7 +1386,7 @@
       <c r="E71" s="5"/>
     </row>
     <row r="72" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B72" s="13"/>
+      <c r="B72" s="16"/>
       <c r="C72" s="5" t="s">
         <v>35</v>
       </c>
@@ -1383,7 +1396,7 @@
       <c r="E72" s="5"/>
     </row>
     <row r="73" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B73" s="13"/>
+      <c r="B73" s="16"/>
       <c r="C73" s="5" t="s">
         <v>79</v>
       </c>
@@ -1393,7 +1406,7 @@
       <c r="E73" s="5"/>
     </row>
     <row r="74" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B74" s="13"/>
+      <c r="B74" s="16"/>
       <c r="C74" s="8" t="s">
         <v>80</v>
       </c>
@@ -1403,7 +1416,7 @@
       <c r="E74" s="5"/>
     </row>
     <row r="75" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B75" s="13"/>
+      <c r="B75" s="16"/>
       <c r="C75" s="8" t="s">
         <v>78</v>
       </c>
@@ -1413,7 +1426,7 @@
       <c r="E75" s="5"/>
     </row>
     <row r="76" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B76" s="13"/>
+      <c r="B76" s="16"/>
       <c r="C76" s="8" t="s">
         <v>77</v>
       </c>
@@ -1423,7 +1436,7 @@
       <c r="E76" s="5"/>
     </row>
     <row r="77" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B77" s="13"/>
+      <c r="B77" s="16"/>
       <c r="C77" s="8" t="s">
         <v>75</v>
       </c>
@@ -1433,7 +1446,7 @@
       <c r="E77" s="5"/>
     </row>
     <row r="78" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B78" s="13"/>
+      <c r="B78" s="16"/>
       <c r="C78" s="8" t="s">
         <v>82</v>
       </c>
@@ -1463,4 +1476,162 @@
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="B1:E15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="1.28515625" customWidth="1"/>
+    <col min="2" max="2" width="20.85546875" customWidth="1"/>
+    <col min="3" max="3" width="25.85546875" customWidth="1"/>
+    <col min="4" max="4" width="18.42578125" customWidth="1"/>
+    <col min="5" max="5" width="20.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B1" s="11"/>
+      <c r="C1" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="2" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B2" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="D2" s="7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B3" s="16"/>
+      <c r="C3" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="D3" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="16"/>
+      <c r="C4" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="D4" s="5">
+        <v>7</v>
+      </c>
+      <c r="E4" s="10"/>
+    </row>
+    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B5" s="16"/>
+      <c r="C5" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="D5" s="5">
+        <v>6</v>
+      </c>
+      <c r="E5" s="10"/>
+    </row>
+    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B6" s="16"/>
+      <c r="C6" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="D6" s="5">
+        <v>8</v>
+      </c>
+      <c r="E6" s="10"/>
+    </row>
+    <row r="7" spans="2:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="16"/>
+      <c r="C7" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7" s="5">
+        <v>8</v>
+      </c>
+      <c r="E7" s="10"/>
+    </row>
+    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B8" s="16"/>
+      <c r="C8" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="D8" s="5">
+        <v>5</v>
+      </c>
+      <c r="E8" s="10"/>
+    </row>
+    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B9" s="16"/>
+      <c r="C9" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="D9" s="5">
+        <v>5</v>
+      </c>
+      <c r="E9" s="10"/>
+    </row>
+    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B10" s="16"/>
+      <c r="C10" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="D10" s="5">
+        <v>3</v>
+      </c>
+      <c r="E10" s="10"/>
+    </row>
+    <row r="11" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B11" s="16"/>
+      <c r="C11" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="D11" s="5">
+        <v>3</v>
+      </c>
+      <c r="E11" s="10"/>
+    </row>
+    <row r="12" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B12" s="16"/>
+      <c r="C12" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="D12" s="5">
+        <v>6</v>
+      </c>
+      <c r="E12" s="10"/>
+    </row>
+    <row r="13" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B13" s="16"/>
+      <c r="C13" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="D13" s="5">
+        <v>2</v>
+      </c>
+      <c r="E13" s="10"/>
+    </row>
+    <row r="14" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B14" s="11"/>
+      <c r="E14" s="10"/>
+    </row>
+    <row r="15" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B15" s="11"/>
+      <c r="E15" s="10"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:B13"/>
+  </mergeCells>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza rota /pedidos com auto-refresh, agrupamento por cliente, imprimir e limpar
</commit_message>
<xml_diff>
--- a/static/cardapio.xlsx
+++ b/static/cardapio.xlsx
@@ -790,7 +790,7 @@
         <v>55</v>
       </c>
       <c r="D4" s="5">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>0</v>
@@ -802,7 +802,7 @@
         <v>25</v>
       </c>
       <c r="D5" s="5">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>1</v>
@@ -814,7 +814,7 @@
         <v>26</v>
       </c>
       <c r="D6" s="5">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>2</v>
@@ -826,7 +826,7 @@
         <v>53</v>
       </c>
       <c r="D7" s="5">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>3</v>
@@ -838,7 +838,7 @@
         <v>52</v>
       </c>
       <c r="D8" s="5">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E8" s="5" t="s">
         <v>4</v>
@@ -850,7 +850,7 @@
         <v>51</v>
       </c>
       <c r="D9" s="5">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E9" s="5" t="s">
         <v>5</v>
@@ -862,7 +862,7 @@
         <v>50</v>
       </c>
       <c r="D10" s="5">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E10" s="5" t="s">
         <v>6</v>
@@ -874,7 +874,7 @@
         <v>56</v>
       </c>
       <c r="D11" s="5">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>7</v>
@@ -886,7 +886,7 @@
         <v>46</v>
       </c>
       <c r="D12" s="5">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>8</v>
@@ -898,7 +898,7 @@
         <v>47</v>
       </c>
       <c r="D13" s="5">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E13" s="5" t="s">
         <v>9</v>
@@ -910,7 +910,7 @@
         <v>48</v>
       </c>
       <c r="D14" s="5">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>10</v>
@@ -922,7 +922,7 @@
         <v>49</v>
       </c>
       <c r="D15" s="5">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E15" s="5" t="s">
         <v>11</v>
@@ -944,7 +944,7 @@
         <v>44</v>
       </c>
       <c r="D17" s="5">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E17" s="5" t="s">
         <v>12</v>
@@ -956,7 +956,7 @@
         <v>43</v>
       </c>
       <c r="D18" s="5">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E18" s="5" t="s">
         <v>13</v>
@@ -968,7 +968,7 @@
         <v>45</v>
       </c>
       <c r="D19" s="5">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E19" s="5" t="s">
         <v>14</v>
@@ -1003,7 +1003,7 @@
         <v>41</v>
       </c>
       <c r="D31" s="5">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E31" s="5"/>
     </row>
@@ -1013,7 +1013,7 @@
         <v>40</v>
       </c>
       <c r="D32" s="5">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E32" s="5"/>
     </row>
@@ -1023,7 +1023,7 @@
         <v>39</v>
       </c>
       <c r="D33" s="5">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E33" s="5"/>
     </row>
@@ -1033,7 +1033,7 @@
         <v>38</v>
       </c>
       <c r="D34" s="5">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E34" s="5"/>
     </row>
@@ -1043,7 +1043,7 @@
         <v>37</v>
       </c>
       <c r="D35" s="5">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E35" s="5"/>
     </row>
@@ -1099,7 +1099,7 @@
         <v>32</v>
       </c>
       <c r="D40" s="5">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E40" s="5" t="s">
         <v>16</v>
@@ -1111,7 +1111,7 @@
         <v>31</v>
       </c>
       <c r="D41" s="5">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E41" s="5" t="s">
         <v>17</v>
@@ -1217,7 +1217,7 @@
         <v>65</v>
       </c>
       <c r="D51" s="5">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E51" s="5"/>
     </row>
@@ -1227,7 +1227,7 @@
         <v>66</v>
       </c>
       <c r="D52" s="5">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E52" s="5"/>
     </row>
@@ -1279,7 +1279,7 @@
         <v>67</v>
       </c>
       <c r="D59" s="5">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E59" s="5"/>
     </row>
@@ -1507,7 +1507,7 @@
         <v>73</v>
       </c>
       <c r="D2" s="7">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="2:5" x14ac:dyDescent="0.25">
@@ -1516,7 +1516,7 @@
         <v>74</v>
       </c>
       <c r="D3" s="5">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1545,7 +1545,7 @@
         <v>81</v>
       </c>
       <c r="D6" s="5">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E6" s="10"/>
     </row>
@@ -1555,7 +1555,7 @@
         <v>35</v>
       </c>
       <c r="D7" s="5">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E7" s="10"/>
     </row>
@@ -1615,7 +1615,7 @@
         <v>82</v>
       </c>
       <c r="D13" s="5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E13" s="10"/>
     </row>

</xml_diff>

<commit_message>
Atualiza planilhas e código com novos pedidos
</commit_message>
<xml_diff>
--- a/static/cardapio.xlsx
+++ b/static/cardapio.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28770" windowHeight="11880" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28770" windowHeight="11880"/>
   </bookViews>
   <sheets>
     <sheet name="Cardapio" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="86">
   <si>
     <t>Pão, hambúrguer, presunto, queijo, bacon, calabresa, ovo frito, frango, coração, alface, tomate, milho, ervilha, batata palha</t>
   </si>
@@ -1334,125 +1334,75 @@
       <c r="E64" s="5"/>
     </row>
     <row r="67" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B67" s="15" t="s">
-        <v>20</v>
-      </c>
-      <c r="C67" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="D67" s="7">
-        <v>5</v>
-      </c>
+      <c r="B67" s="15"/>
+      <c r="C67" s="6"/>
+      <c r="D67" s="7"/>
       <c r="E67" s="5"/>
     </row>
     <row r="68" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B68" s="16"/>
-      <c r="C68" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="D68" s="5">
-        <v>5</v>
-      </c>
+      <c r="C68" s="5"/>
+      <c r="D68" s="5"/>
       <c r="E68" s="5"/>
     </row>
     <row r="69" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B69" s="16"/>
-      <c r="C69" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="D69" s="5">
-        <v>7</v>
-      </c>
+      <c r="C69" s="5"/>
+      <c r="D69" s="5"/>
       <c r="E69" s="5"/>
     </row>
     <row r="70" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B70" s="16"/>
-      <c r="C70" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="D70" s="5">
-        <v>6</v>
-      </c>
+      <c r="C70" s="5"/>
+      <c r="D70" s="5"/>
       <c r="E70" s="5"/>
     </row>
     <row r="71" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B71" s="16"/>
-      <c r="C71" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="D71" s="5">
-        <v>8</v>
-      </c>
+      <c r="C71" s="5"/>
+      <c r="D71" s="5"/>
       <c r="E71" s="5"/>
     </row>
     <row r="72" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B72" s="16"/>
-      <c r="C72" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="D72" s="5">
-        <v>8</v>
-      </c>
+      <c r="C72" s="5"/>
+      <c r="D72" s="5"/>
       <c r="E72" s="5"/>
     </row>
     <row r="73" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B73" s="16"/>
-      <c r="C73" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="D73" s="5">
-        <v>5</v>
-      </c>
+      <c r="C73" s="5"/>
+      <c r="D73" s="5"/>
       <c r="E73" s="5"/>
     </row>
     <row r="74" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B74" s="16"/>
-      <c r="C74" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="D74" s="5">
-        <v>5</v>
-      </c>
+      <c r="C74" s="8"/>
+      <c r="D74" s="5"/>
       <c r="E74" s="5"/>
     </row>
     <row r="75" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B75" s="16"/>
-      <c r="C75" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="D75" s="5">
-        <v>3</v>
-      </c>
+      <c r="C75" s="8"/>
+      <c r="D75" s="5"/>
       <c r="E75" s="5"/>
     </row>
     <row r="76" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B76" s="16"/>
-      <c r="C76" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="D76" s="5">
-        <v>3</v>
-      </c>
+      <c r="C76" s="8"/>
+      <c r="D76" s="5"/>
       <c r="E76" s="5"/>
     </row>
     <row r="77" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B77" s="16"/>
-      <c r="C77" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="D77" s="5">
-        <v>6</v>
-      </c>
+      <c r="C77" s="8"/>
+      <c r="D77" s="5"/>
       <c r="E77" s="5"/>
     </row>
     <row r="78" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B78" s="16"/>
-      <c r="C78" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="D78" s="5">
-        <v>2</v>
-      </c>
+      <c r="C78" s="8"/>
+      <c r="D78" s="5"/>
       <c r="E78" s="5"/>
     </row>
   </sheetData>

</xml_diff>